<commit_message>
Add Dkckerfile for Render deplotment
</commit_message>
<xml_diff>
--- a/backend/megadata/Price Lease_Well List_2.5 Miles Radius_TRRC.xlsx
+++ b/backend/megadata/Price Lease_Well List_2.5 Miles Radius_TRRC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gxia\Python\Saguaro_Petroleum_Well_Production_Management\backend\megadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gxia\Python\SP_Petroleum_Well_Production_Management\backend\megadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C943AC0A-152B-417F-B1A1-27AF854ADB37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3432EFDD-9510-4AA5-8C86-4A9E9CA4C471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14310" yWindow="0" windowWidth="14580" windowHeight="17370" xr2:uid="{A0A74406-5AD6-430F-B3D8-A5577271F83F}"/>
+    <workbookView xWindow="-28740" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{A0A74406-5AD6-430F-B3D8-A5577271F83F}"/>
   </bookViews>
   <sheets>
     <sheet name="2.5 Miles Radius" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4924" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4925" uniqueCount="375">
   <si>
     <t>API</t>
   </si>
@@ -1157,12 +1157,15 @@
   <si>
     <t xml:space="preserve">8-1 </t>
   </si>
+  <si>
+    <t>9-3W</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1306,6 +1309,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1670,7 +1681,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1691,6 +1702,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2070,50 +2082,50 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:AO401"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="13.1796875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7265625" customWidth="1"/>
-    <col min="7" max="7" width="63.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.453125" customWidth="1"/>
-    <col min="9" max="9" width="18.1796875" customWidth="1"/>
+    <col min="1" max="2" width="13.140625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="63.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="29.140625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="31" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="27" customWidth="1"/>
-    <col min="17" max="17" width="11.81640625" customWidth="1"/>
-    <col min="18" max="18" width="16.54296875" customWidth="1"/>
-    <col min="19" max="19" width="8.453125" customWidth="1"/>
-    <col min="20" max="20" width="30.26953125" customWidth="1"/>
-    <col min="21" max="21" width="5.81640625" customWidth="1"/>
-    <col min="22" max="22" width="7.81640625" customWidth="1"/>
+    <col min="17" max="17" width="11.85546875" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" customWidth="1"/>
+    <col min="19" max="19" width="8.42578125" customWidth="1"/>
+    <col min="20" max="20" width="30.28515625" customWidth="1"/>
+    <col min="21" max="21" width="5.85546875" customWidth="1"/>
+    <col min="22" max="22" width="7.85546875" customWidth="1"/>
     <col min="23" max="23" width="10" customWidth="1"/>
     <col min="24" max="24" width="12" customWidth="1"/>
     <col min="25" max="25" width="10" customWidth="1"/>
     <col min="26" max="26" width="12" customWidth="1"/>
-    <col min="27" max="27" width="18.81640625" customWidth="1"/>
-    <col min="28" max="28" width="7.7265625" customWidth="1"/>
-    <col min="29" max="29" width="8.26953125" customWidth="1"/>
-    <col min="30" max="30" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="32.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.85546875" customWidth="1"/>
+    <col min="28" max="28" width="7.7109375" customWidth="1"/>
+    <col min="29" max="29" width="8.28515625" customWidth="1"/>
+    <col min="30" max="30" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="27" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="30.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="18.453125" style="7" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="17.7265625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="18.42578125" style="7" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="31" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" s="2" customFormat="1" ht="16" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:41" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -2238,7 +2250,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>105</v>
       </c>
@@ -2280,7 +2292,7 @@
         <v>105___1</v>
       </c>
     </row>
-    <row r="3" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>105</v>
       </c>
@@ -2322,7 +2334,7 @@
         <v>105___1</v>
       </c>
     </row>
-    <row r="4" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>105</v>
       </c>
@@ -2364,7 +2376,7 @@
         <v>105___2</v>
       </c>
     </row>
-    <row r="5" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>10500836</v>
       </c>
@@ -2452,7 +2464,7 @@
         <v>5303</v>
       </c>
     </row>
-    <row r="6" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>10500836</v>
       </c>
@@ -2537,7 +2549,7 @@
         <v>5303</v>
       </c>
     </row>
-    <row r="7" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>10500836</v>
       </c>
@@ -2625,7 +2637,7 @@
         <v>5303</v>
       </c>
     </row>
-    <row r="8" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>10500836</v>
       </c>
@@ -2713,7 +2725,7 @@
         <v>5303</v>
       </c>
     </row>
-    <row r="9" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>10500836</v>
       </c>
@@ -2801,7 +2813,7 @@
         <v>5303</v>
       </c>
     </row>
-    <row r="10" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>10500837</v>
       </c>
@@ -2886,7 +2898,7 @@
         <v>5570</v>
       </c>
     </row>
-    <row r="11" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10500837</v>
       </c>
@@ -2974,7 +2986,7 @@
         <v>5570</v>
       </c>
     </row>
-    <row r="12" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>10500837</v>
       </c>
@@ -3062,7 +3074,7 @@
         <v>5570</v>
       </c>
     </row>
-    <row r="13" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>10500838</v>
       </c>
@@ -3144,7 +3156,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>10500838</v>
       </c>
@@ -3226,7 +3238,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>10500838</v>
       </c>
@@ -3308,7 +3320,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>10500839</v>
       </c>
@@ -3426,7 +3438,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>10500839</v>
       </c>
@@ -3541,7 +3553,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>10500839</v>
       </c>
@@ -3659,7 +3671,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>10500839</v>
       </c>
@@ -3777,7 +3789,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>10500839</v>
       </c>
@@ -3895,7 +3907,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>10500839</v>
       </c>
@@ -4013,7 +4025,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>10500839</v>
       </c>
@@ -4131,7 +4143,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>10501196</v>
       </c>
@@ -4219,7 +4231,7 @@
         <v>5600</v>
       </c>
     </row>
-    <row r="24" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>10501196</v>
       </c>
@@ -4307,7 +4319,7 @@
         <v>5600</v>
       </c>
     </row>
-    <row r="25" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>10501197</v>
       </c>
@@ -4395,7 +4407,7 @@
         <v>5230</v>
       </c>
     </row>
-    <row r="26" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>10501197</v>
       </c>
@@ -4483,7 +4495,7 @@
         <v>5230</v>
       </c>
     </row>
-    <row r="27" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>10501198</v>
       </c>
@@ -4565,7 +4577,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>10501198</v>
       </c>
@@ -4647,7 +4659,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="29" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>10501199</v>
       </c>
@@ -4735,7 +4747,7 @@
         <v>5260</v>
       </c>
     </row>
-    <row r="30" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>10501199</v>
       </c>
@@ -4823,7 +4835,7 @@
         <v>5260</v>
       </c>
     </row>
-    <row r="31" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>10501938</v>
       </c>
@@ -4911,7 +4923,7 @@
         <v>5400</v>
       </c>
     </row>
-    <row r="32" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>10501938</v>
       </c>
@@ -4996,7 +5008,7 @@
         <v>5400</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>10501938</v>
       </c>
@@ -5084,7 +5096,7 @@
         <v>5400</v>
       </c>
     </row>
-    <row r="34" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>10502537</v>
       </c>
@@ -5166,7 +5178,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="35" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>10502537</v>
       </c>
@@ -5248,7 +5260,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="36" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>10502537</v>
       </c>
@@ -5330,7 +5342,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="37" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>10502538</v>
       </c>
@@ -5412,7 +5424,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="38" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>10502538</v>
       </c>
@@ -5494,7 +5506,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>10502538</v>
       </c>
@@ -5576,7 +5588,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="40" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>10502539</v>
       </c>
@@ -5658,7 +5670,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="41" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>10502539</v>
       </c>
@@ -5740,7 +5752,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="42" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>10502540</v>
       </c>
@@ -5822,7 +5834,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="43" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>10502540</v>
       </c>
@@ -5904,7 +5916,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="44" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>10502547</v>
       </c>
@@ -5986,7 +5998,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>10502547</v>
       </c>
@@ -6068,7 +6080,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="46" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>10502552</v>
       </c>
@@ -6150,7 +6162,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="47" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>10502552</v>
       </c>
@@ -6232,7 +6244,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>10502552</v>
       </c>
@@ -6314,7 +6326,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="49" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>10502552</v>
       </c>
@@ -6396,7 +6408,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>10502552</v>
       </c>
@@ -6478,7 +6490,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="51" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>10502556</v>
       </c>
@@ -6560,7 +6572,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>10502556</v>
       </c>
@@ -6642,7 +6654,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="53" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>10502556</v>
       </c>
@@ -6724,7 +6736,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>10502556</v>
       </c>
@@ -6806,7 +6818,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="55" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>10502556</v>
       </c>
@@ -6888,7 +6900,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="56" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>10502560</v>
       </c>
@@ -6970,7 +6982,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="57" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>10502560</v>
       </c>
@@ -7052,7 +7064,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="58" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>10502560</v>
       </c>
@@ -7134,7 +7146,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="59" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>10502560</v>
       </c>
@@ -7216,7 +7228,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="60" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>10502564</v>
       </c>
@@ -7298,7 +7310,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="61" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>10502564</v>
       </c>
@@ -7380,7 +7392,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="62" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>10502564</v>
       </c>
@@ -7462,7 +7474,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="63" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>10502564</v>
       </c>
@@ -7544,7 +7556,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="64" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>10502568</v>
       </c>
@@ -7632,7 +7644,7 @@
         <v>5290</v>
       </c>
     </row>
-    <row r="65" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>10502568</v>
       </c>
@@ -7720,7 +7732,7 @@
         <v>5290</v>
       </c>
     </row>
-    <row r="66" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>10502570</v>
       </c>
@@ -7802,7 +7814,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="67" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>10502570</v>
       </c>
@@ -7884,7 +7896,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="68" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>10502572</v>
       </c>
@@ -7966,7 +7978,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="69" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>10502575</v>
       </c>
@@ -8054,7 +8066,7 @@
         <v>5326</v>
       </c>
     </row>
-    <row r="70" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>10502578</v>
       </c>
@@ -8136,7 +8148,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="71" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>10502578</v>
       </c>
@@ -8218,7 +8230,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="72" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>10502580</v>
       </c>
@@ -8300,7 +8312,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="73" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>10502580</v>
       </c>
@@ -8382,7 +8394,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="74" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>10502580</v>
       </c>
@@ -8464,7 +8476,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>10502582</v>
       </c>
@@ -8546,7 +8558,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="76" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>10502582</v>
       </c>
@@ -8628,7 +8640,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="77" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>10502583</v>
       </c>
@@ -8716,7 +8728,7 @@
         <v>5420</v>
       </c>
     </row>
-    <row r="78" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>10502583</v>
       </c>
@@ -8804,7 +8816,7 @@
         <v>5420</v>
       </c>
     </row>
-    <row r="79" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>10502583</v>
       </c>
@@ -8892,7 +8904,7 @@
         <v>5420</v>
       </c>
     </row>
-    <row r="80" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>10502583</v>
       </c>
@@ -8980,7 +8992,7 @@
         <v>5420</v>
       </c>
     </row>
-    <row r="81" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>10502584</v>
       </c>
@@ -9062,7 +9074,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="82" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>10502584</v>
       </c>
@@ -9144,7 +9156,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="83" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>10502585</v>
       </c>
@@ -9226,7 +9238,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="84" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>10502585</v>
       </c>
@@ -9308,7 +9320,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="85" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>10502585</v>
       </c>
@@ -9390,7 +9402,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="86" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>10502586</v>
       </c>
@@ -9472,7 +9484,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="87" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>10502586</v>
       </c>
@@ -9554,7 +9566,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="88" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>10502586</v>
       </c>
@@ -9636,7 +9648,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="89" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>10502586</v>
       </c>
@@ -9718,7 +9730,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="90" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>10502591</v>
       </c>
@@ -9800,7 +9812,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="91" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>10502591</v>
       </c>
@@ -9882,7 +9894,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="92" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>10502591</v>
       </c>
@@ -9964,7 +9976,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="93" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>10502593</v>
       </c>
@@ -10046,7 +10058,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="94" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>10502593</v>
       </c>
@@ -10128,7 +10140,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="95" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>10502594</v>
       </c>
@@ -10210,7 +10222,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="96" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>10502594</v>
       </c>
@@ -10292,7 +10304,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="97" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>10502597</v>
       </c>
@@ -10374,7 +10386,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="98" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>10502597</v>
       </c>
@@ -10456,7 +10468,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="99" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>10502597</v>
       </c>
@@ -10538,7 +10550,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="100" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>10502597</v>
       </c>
@@ -10620,7 +10632,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="101" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>10502597</v>
       </c>
@@ -10702,7 +10714,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="102" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>10502598</v>
       </c>
@@ -10784,7 +10796,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="103" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>10502598</v>
       </c>
@@ -10866,7 +10878,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="104" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>10502598</v>
       </c>
@@ -10948,7 +10960,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="105" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>10502599</v>
       </c>
@@ -11030,7 +11042,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="106" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>10502599</v>
       </c>
@@ -11112,7 +11124,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="107" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>10502599</v>
       </c>
@@ -11194,7 +11206,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="108" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>10502599</v>
       </c>
@@ -11276,7 +11288,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="109" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>10502600</v>
       </c>
@@ -11358,7 +11370,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="110" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>10502600</v>
       </c>
@@ -11440,7 +11452,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="111" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>10502600</v>
       </c>
@@ -11522,7 +11534,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="112" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>10502600</v>
       </c>
@@ -11604,7 +11616,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="113" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>10502601</v>
       </c>
@@ -11686,7 +11698,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="114" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>10502601</v>
       </c>
@@ -11768,7 +11780,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="115" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>10502601</v>
       </c>
@@ -11850,7 +11862,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="116" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>10502601</v>
       </c>
@@ -11932,7 +11944,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="117" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>10502601</v>
       </c>
@@ -12014,7 +12026,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="118" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>10502601</v>
       </c>
@@ -12096,7 +12108,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="119" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>10502602</v>
       </c>
@@ -12178,7 +12190,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="120" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>10502602</v>
       </c>
@@ -12260,7 +12272,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="121" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>10502603</v>
       </c>
@@ -12348,7 +12360,7 @@
         <v>5216</v>
       </c>
     </row>
-    <row r="122" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>10502603</v>
       </c>
@@ -12436,7 +12448,7 @@
         <v>5216</v>
       </c>
     </row>
-    <row r="123" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>10502603</v>
       </c>
@@ -12524,7 +12536,7 @@
         <v>5216</v>
       </c>
     </row>
-    <row r="124" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
         <v>10502603</v>
       </c>
@@ -12612,7 +12624,7 @@
         <v>5216</v>
       </c>
     </row>
-    <row r="125" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A125" s="3">
         <v>10502604</v>
       </c>
@@ -12694,7 +12706,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="126" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A126" s="3">
         <v>10502604</v>
       </c>
@@ -12776,7 +12788,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="127" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A127" s="3">
         <v>10502604</v>
       </c>
@@ -12858,7 +12870,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="128" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A128" s="3">
         <v>10502604</v>
       </c>
@@ -12940,7 +12952,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="129" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A129" s="3">
         <v>10502604</v>
       </c>
@@ -13022,7 +13034,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="130" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A130" s="3">
         <v>10502604</v>
       </c>
@@ -13104,7 +13116,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="131" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A131" s="3">
         <v>10502605</v>
       </c>
@@ -13186,7 +13198,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="132" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A132" s="3">
         <v>10502605</v>
       </c>
@@ -13268,7 +13280,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="133" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A133" s="3">
         <v>10502606</v>
       </c>
@@ -13350,7 +13362,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="134" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A134" s="3">
         <v>10502606</v>
       </c>
@@ -13432,7 +13444,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="135" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A135" s="3">
         <v>10502606</v>
       </c>
@@ -13514,7 +13526,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="136" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A136" s="3">
         <v>10502606</v>
       </c>
@@ -13596,7 +13608,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="137" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A137" s="3">
         <v>10502607</v>
       </c>
@@ -13678,7 +13690,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="138" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A138" s="3">
         <v>10502607</v>
       </c>
@@ -13760,7 +13772,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="139" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A139" s="3">
         <v>10502607</v>
       </c>
@@ -13842,7 +13854,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="140" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A140" s="3">
         <v>10502607</v>
       </c>
@@ -13924,7 +13936,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="141" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A141" s="3">
         <v>10502607</v>
       </c>
@@ -14006,7 +14018,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="142" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A142" s="3">
         <v>10502608</v>
       </c>
@@ -14088,7 +14100,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="143" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A143" s="3">
         <v>10502608</v>
       </c>
@@ -14167,7 +14179,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="144" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A144" s="3">
         <v>10502608</v>
       </c>
@@ -14249,7 +14261,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="145" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A145" s="3">
         <v>10502608</v>
       </c>
@@ -14331,7 +14343,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="146" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A146" s="3">
         <v>10502608</v>
       </c>
@@ -14413,7 +14425,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="147" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A147" s="3">
         <v>10502608</v>
       </c>
@@ -14495,7 +14507,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="148" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A148" s="3">
         <v>10502609</v>
       </c>
@@ -14577,7 +14589,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="149" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A149" s="3">
         <v>10502609</v>
       </c>
@@ -14659,7 +14671,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="150" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A150" s="3">
         <v>10502609</v>
       </c>
@@ -14741,7 +14753,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="151" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A151" s="3">
         <v>10502609</v>
       </c>
@@ -14823,7 +14835,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="152" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A152" s="3">
         <v>10503108</v>
       </c>
@@ -14911,7 +14923,7 @@
         <v>5654</v>
       </c>
     </row>
-    <row r="153" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A153" s="3">
         <v>10503109</v>
       </c>
@@ -14993,7 +15005,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="154" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A154" s="3">
         <v>10503111</v>
       </c>
@@ -15081,7 +15093,7 @@
         <v>5680</v>
       </c>
     </row>
-    <row r="155" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A155" s="3">
         <v>10503111</v>
       </c>
@@ -15169,7 +15181,7 @@
         <v>5680</v>
       </c>
     </row>
-    <row r="156" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A156" s="3">
         <v>10503112</v>
       </c>
@@ -15257,7 +15269,7 @@
         <v>5642</v>
       </c>
     </row>
-    <row r="157" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A157" s="3">
         <v>10503112</v>
       </c>
@@ -15345,7 +15357,7 @@
         <v>5642</v>
       </c>
     </row>
-    <row r="158" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A158" s="3">
         <v>10503114</v>
       </c>
@@ -15408,7 +15420,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="159" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A159" s="3">
         <v>10503465</v>
       </c>
@@ -15496,7 +15508,7 @@
         <v>5529</v>
       </c>
     </row>
-    <row r="160" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A160" s="3">
         <v>10503465</v>
       </c>
@@ -15584,7 +15596,7 @@
         <v>5529</v>
       </c>
     </row>
-    <row r="161" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A161" s="3">
         <v>10510147</v>
       </c>
@@ -15672,7 +15684,7 @@
         <v>5380</v>
       </c>
     </row>
-    <row r="162" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A162" s="3">
         <v>10510147</v>
       </c>
@@ -15760,7 +15772,7 @@
         <v>5380</v>
       </c>
     </row>
-    <row r="163" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A163" s="3">
         <v>10510147</v>
       </c>
@@ -15848,7 +15860,7 @@
         <v>5380</v>
       </c>
     </row>
-    <row r="164" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A164" s="3">
         <v>10510148</v>
       </c>
@@ -15936,7 +15948,7 @@
         <v>5085</v>
       </c>
     </row>
-    <row r="165" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A165" s="3">
         <v>10510148</v>
       </c>
@@ -16024,7 +16036,7 @@
         <v>5085</v>
       </c>
     </row>
-    <row r="166" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A166" s="3">
         <v>10510148</v>
       </c>
@@ -16112,7 +16124,7 @@
         <v>5085</v>
       </c>
     </row>
-    <row r="167" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A167" s="3">
         <v>10510148</v>
       </c>
@@ -16200,7 +16212,7 @@
         <v>5085</v>
       </c>
     </row>
-    <row r="168" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A168" s="3">
         <v>10510150</v>
       </c>
@@ -16282,7 +16294,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="169" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A169" s="3">
         <v>10510150</v>
       </c>
@@ -16364,7 +16376,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="170" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A170" s="3">
         <v>10510153</v>
       </c>
@@ -16446,7 +16458,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="171" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A171" s="3">
         <v>10510153</v>
       </c>
@@ -16528,7 +16540,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="172" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A172" s="3">
         <v>10510153</v>
       </c>
@@ -16610,7 +16622,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="173" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A173" s="3">
         <v>10510153</v>
       </c>
@@ -16692,7 +16704,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="174" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A174" s="3">
         <v>10510153</v>
       </c>
@@ -16774,7 +16786,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="175" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A175" s="3">
         <v>10510153</v>
       </c>
@@ -16856,7 +16868,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="176" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A176" s="3">
         <v>10510153</v>
       </c>
@@ -16938,7 +16950,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="177" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A177" s="3">
         <v>10510154</v>
       </c>
@@ -17020,7 +17032,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="178" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A178" s="3">
         <v>10510154</v>
       </c>
@@ -17102,7 +17114,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="179" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A179" s="3">
         <v>10510154</v>
       </c>
@@ -17184,7 +17196,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="180" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A180" s="3">
         <v>10510155</v>
       </c>
@@ -17266,7 +17278,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="181" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A181" s="3">
         <v>10510155</v>
       </c>
@@ -17348,7 +17360,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="182" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A182" s="3">
         <v>10510156</v>
       </c>
@@ -17430,7 +17442,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="183" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A183" s="3">
         <v>10510156</v>
       </c>
@@ -17512,7 +17524,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="184" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A184" s="3">
         <v>10510265</v>
       </c>
@@ -17575,7 +17587,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="185" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A185" s="3">
         <v>10510279</v>
       </c>
@@ -17657,7 +17669,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="186" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A186" s="3">
         <v>10510279</v>
       </c>
@@ -17739,7 +17751,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="187" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A187" s="3">
         <v>10510280</v>
       </c>
@@ -17821,7 +17833,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="188" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A188" s="3">
         <v>10510280</v>
       </c>
@@ -17903,7 +17915,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="189" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A189" s="3">
         <v>10510281</v>
       </c>
@@ -18027,7 +18039,7 @@
         <v>7126</v>
       </c>
     </row>
-    <row r="190" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A190" s="3">
         <v>10510281</v>
       </c>
@@ -18151,7 +18163,7 @@
         <v>7126</v>
       </c>
     </row>
-    <row r="191" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A191" s="3">
         <v>10510282</v>
       </c>
@@ -18233,7 +18245,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="192" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A192" s="3">
         <v>10510298</v>
       </c>
@@ -18315,7 +18327,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="193" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A193" s="3">
         <v>10510298</v>
       </c>
@@ -18397,7 +18409,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="194" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A194" s="3">
         <v>10510298</v>
       </c>
@@ -18479,7 +18491,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="195" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A195" s="3">
         <v>10510298</v>
       </c>
@@ -18561,7 +18573,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="196" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A196" s="3">
         <v>10510301</v>
       </c>
@@ -18643,7 +18655,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="197" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A197" s="3">
         <v>10510301</v>
       </c>
@@ -18725,7 +18737,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="198" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A198" s="3">
         <v>10510301</v>
       </c>
@@ -18807,7 +18819,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="199" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A199" s="3">
         <v>10510409</v>
       </c>
@@ -18886,7 +18898,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="200" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A200" s="3">
         <v>10510409</v>
       </c>
@@ -18968,7 +18980,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="201" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A201" s="3">
         <v>10534153</v>
       </c>
@@ -19086,7 +19098,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="202" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A202" s="3">
         <v>10534153</v>
       </c>
@@ -19204,7 +19216,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="203" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A203" s="3">
         <v>10534154</v>
       </c>
@@ -19298,7 +19310,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="204" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A204" s="3">
         <v>10534161</v>
       </c>
@@ -19392,7 +19404,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="205" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A205" s="3">
         <v>10535606</v>
       </c>
@@ -19510,7 +19522,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="206" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A206" s="3">
         <v>10535606</v>
       </c>
@@ -19628,7 +19640,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="207" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A207" s="3">
         <v>10535606</v>
       </c>
@@ -19746,7 +19758,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="208" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A208" s="3">
         <v>10535646</v>
       </c>
@@ -19864,7 +19876,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="209" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A209" s="3">
         <v>10535647</v>
       </c>
@@ -19979,7 +19991,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="210" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A210" s="3">
         <v>10535868</v>
       </c>
@@ -20099,7 +20111,7 @@
         <v>5573</v>
       </c>
     </row>
-    <row r="211" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A211" s="3">
         <v>10535868</v>
       </c>
@@ -20220,7 +20232,7 @@
         <v>5573</v>
       </c>
     </row>
-    <row r="212" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A212" s="3">
         <v>10535934</v>
       </c>
@@ -20340,7 +20352,7 @@
         <v>5543</v>
       </c>
     </row>
-    <row r="213" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A213" s="3">
         <v>10535944</v>
       </c>
@@ -20463,7 +20475,7 @@
         <v>5470</v>
       </c>
     </row>
-    <row r="214" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A214" s="3">
         <v>10535977</v>
       </c>
@@ -20562,7 +20574,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="215" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A215" s="3">
         <v>10536001</v>
       </c>
@@ -20682,7 +20694,7 @@
         <v>5550</v>
       </c>
     </row>
-    <row r="216" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A216" s="3">
         <v>10536001</v>
       </c>
@@ -20802,7 +20814,7 @@
         <v>5550</v>
       </c>
     </row>
-    <row r="217" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A217" s="3">
         <v>10536046</v>
       </c>
@@ -20889,7 +20901,7 @@
         <v>10536046___2</v>
       </c>
     </row>
-    <row r="218" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A218" s="3">
         <v>10537515</v>
       </c>
@@ -21007,7 +21019,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="219" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A219" s="3">
         <v>10537659</v>
       </c>
@@ -21125,7 +21137,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="220" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A220" s="3">
         <v>10538300</v>
       </c>
@@ -21243,7 +21255,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="221" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A221" s="3">
         <v>10538482</v>
       </c>
@@ -21361,7 +21373,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="222" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A222" s="3">
         <v>10538483</v>
       </c>
@@ -21479,7 +21491,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="223" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A223" s="3">
         <v>10538685</v>
       </c>
@@ -21597,7 +21609,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="224" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A224" s="3">
         <v>10538786</v>
       </c>
@@ -21696,7 +21708,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="225" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A225" s="3">
         <v>10539056</v>
       </c>
@@ -21814,7 +21826,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="226" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A226" s="3">
         <v>10539057</v>
       </c>
@@ -21932,7 +21944,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="227" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A227" s="3">
         <v>10539315</v>
       </c>
@@ -22050,7 +22062,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="228" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A228" s="3">
         <v>10539316</v>
       </c>
@@ -22168,7 +22180,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="229" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A229" s="3">
         <v>10539317</v>
       </c>
@@ -22286,7 +22298,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="230" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A230" s="3">
         <v>10539423</v>
       </c>
@@ -22404,7 +22416,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="231" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A231" s="3">
         <v>10539591</v>
       </c>
@@ -22522,7 +22534,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="232" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A232" s="3">
         <v>10539592</v>
       </c>
@@ -22640,7 +22652,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="233" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A233" s="3">
         <v>10539619</v>
       </c>
@@ -22758,7 +22770,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="234" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A234" s="3">
         <v>10539620</v>
       </c>
@@ -22876,7 +22888,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="235" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A235" s="3">
         <v>10539621</v>
       </c>
@@ -22975,7 +22987,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="236" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A236" s="3">
         <v>10539621</v>
       </c>
@@ -23068,7 +23080,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="237" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A237" s="3">
         <v>10539622</v>
       </c>
@@ -23186,7 +23198,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="238" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A238" s="3">
         <v>10539966</v>
       </c>
@@ -23304,7 +23316,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="239" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A239" s="3">
         <v>10540212</v>
       </c>
@@ -23422,7 +23434,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="240" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A240" s="3">
         <v>10540213</v>
       </c>
@@ -23540,7 +23552,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="241" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A241" s="3">
         <v>10540214</v>
       </c>
@@ -23658,7 +23670,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="242" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A242" s="3">
         <v>10540225</v>
       </c>
@@ -23776,7 +23788,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="243" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A243" s="3">
         <v>10540226</v>
       </c>
@@ -23863,7 +23875,7 @@
         <v>10540226___246</v>
       </c>
     </row>
-    <row r="244" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A244" s="3">
         <v>10540537</v>
       </c>
@@ -23981,7 +23993,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="245" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A245" s="3">
         <v>10540538</v>
       </c>
@@ -24099,7 +24111,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="246" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A246" s="3">
         <v>10540540</v>
       </c>
@@ -24217,7 +24229,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="247" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A247" s="3">
         <v>10540541</v>
       </c>
@@ -24335,7 +24347,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="248" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A248" s="3">
         <v>10540939</v>
       </c>
@@ -24453,7 +24465,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="249" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A249" s="3">
         <v>10541021</v>
       </c>
@@ -24571,7 +24583,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="250" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A250" s="3">
         <v>10541022</v>
       </c>
@@ -24689,7 +24701,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="251" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A251" s="3">
         <v>10541852</v>
       </c>
@@ -24807,7 +24819,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="252" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A252" s="3">
         <v>10541853</v>
       </c>
@@ -24925,7 +24937,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="253" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A253" s="3">
         <v>10541858</v>
       </c>
@@ -25043,7 +25055,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="254" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A254" s="3">
         <v>10542051</v>
       </c>
@@ -25161,7 +25173,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="255" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A255" s="3">
         <v>10542051</v>
       </c>
@@ -25273,7 +25285,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="256" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A256" s="3">
         <v>10542052</v>
       </c>
@@ -25391,7 +25403,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="257" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A257" s="3">
         <v>10542476</v>
       </c>
@@ -25509,7 +25521,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="258" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A258" s="3">
         <v>10542477</v>
       </c>
@@ -25627,7 +25639,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="259" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A259" s="3">
         <v>10542483</v>
       </c>
@@ -25745,7 +25757,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="260" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A260" s="3">
         <v>10542484</v>
       </c>
@@ -25863,7 +25875,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="261" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A261" s="3">
         <v>371</v>
       </c>
@@ -25905,7 +25917,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="262" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A262" s="3">
         <v>371</v>
       </c>
@@ -25947,7 +25959,7 @@
         <v>371___1A</v>
       </c>
     </row>
-    <row r="263" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A263" s="3">
         <v>371</v>
       </c>
@@ -25989,7 +26001,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="264" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A264" s="3">
         <v>371</v>
       </c>
@@ -26031,7 +26043,7 @@
         <v>371___2B</v>
       </c>
     </row>
-    <row r="265" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A265" s="3">
         <v>371</v>
       </c>
@@ -26073,7 +26085,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="266" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A266" s="3">
         <v>371</v>
       </c>
@@ -26115,7 +26127,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="267" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A267" s="3">
         <v>371</v>
       </c>
@@ -26157,7 +26169,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="268" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A268" s="3">
         <v>371</v>
       </c>
@@ -26199,7 +26211,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="269" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A269" s="3">
         <v>371</v>
       </c>
@@ -26241,7 +26253,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="270" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A270" s="3">
         <v>371</v>
       </c>
@@ -26283,7 +26295,7 @@
         <v>371___2D</v>
       </c>
     </row>
-    <row r="271" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A271" s="3">
         <v>371</v>
       </c>
@@ -26325,7 +26337,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="272" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A272" s="3">
         <v>371</v>
       </c>
@@ -26367,7 +26379,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="273" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A273" s="3">
         <v>371</v>
       </c>
@@ -26409,7 +26421,7 @@
         <v>371___2</v>
       </c>
     </row>
-    <row r="274" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A274" s="3">
         <v>371</v>
       </c>
@@ -26451,7 +26463,7 @@
         <v>371___1</v>
       </c>
     </row>
-    <row r="275" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A275" s="3">
         <v>37100537</v>
       </c>
@@ -26530,7 +26542,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="276" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A276" s="3">
         <v>37100538</v>
       </c>
@@ -26619,7 +26631,7 @@
         <v>5192</v>
       </c>
     </row>
-    <row r="277" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A277" s="3">
         <v>37100538</v>
       </c>
@@ -26704,7 +26716,7 @@
         <v>5192</v>
       </c>
     </row>
-    <row r="278" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A278" s="3">
         <v>37101754</v>
       </c>
@@ -26792,7 +26804,7 @@
         <v>5595</v>
       </c>
     </row>
-    <row r="279" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A279" s="3">
         <v>37104300</v>
       </c>
@@ -26880,7 +26892,7 @@
         <v>5100</v>
       </c>
     </row>
-    <row r="280" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A280" s="3">
         <v>37104301</v>
       </c>
@@ -26956,7 +26968,7 @@
         <v>5115</v>
       </c>
     </row>
-    <row r="281" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A281" s="3">
         <v>37104301</v>
       </c>
@@ -27044,7 +27056,7 @@
         <v>5115</v>
       </c>
     </row>
-    <row r="282" spans="1:39" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:39" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A282" s="4">
         <v>37104303</v>
       </c>
@@ -27162,7 +27174,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="283" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A283" s="3">
         <v>37104303</v>
       </c>
@@ -27279,7 +27291,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="284" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A284" s="3">
         <v>37104303</v>
       </c>
@@ -27396,7 +27408,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="285" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A285" s="3">
         <v>37104303</v>
       </c>
@@ -27513,7 +27525,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="286" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A286" s="3">
         <v>37104303</v>
       </c>
@@ -27630,7 +27642,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="287" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A287" s="3">
         <v>37104304</v>
       </c>
@@ -27706,7 +27718,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="288" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A288" s="3">
         <v>37104304</v>
       </c>
@@ -27788,7 +27800,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="289" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A289" s="3">
         <v>37104304</v>
       </c>
@@ -27870,7 +27882,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="290" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A290" s="3">
         <v>37104921</v>
       </c>
@@ -27952,7 +27964,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="291" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A291" s="3">
         <v>37104921</v>
       </c>
@@ -28034,7 +28046,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="292" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A292" s="3">
         <v>37104922</v>
       </c>
@@ -28116,7 +28128,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="293" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A293" s="3">
         <v>37104923</v>
       </c>
@@ -28195,7 +28207,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="294" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A294" s="3">
         <v>37104923</v>
       </c>
@@ -28277,7 +28289,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="295" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A295" s="3">
         <v>37104924</v>
       </c>
@@ -28359,7 +28371,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="296" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A296" s="3">
         <v>37110038</v>
       </c>
@@ -28483,7 +28495,7 @@
         <v>5350</v>
       </c>
     </row>
-    <row r="297" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A297" s="3">
         <v>37130139</v>
       </c>
@@ -28601,7 +28613,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="298" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A298" s="3">
         <v>37130189</v>
       </c>
@@ -28716,7 +28728,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="299" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A299" s="3">
         <v>37130189</v>
       </c>
@@ -28828,7 +28840,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="300" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A300" s="3">
         <v>37130189</v>
       </c>
@@ -28940,7 +28952,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="301" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A301" s="3">
         <v>37130189</v>
       </c>
@@ -29055,7 +29067,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="302" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A302" s="3">
         <v>37130189</v>
       </c>
@@ -29170,7 +29182,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="303" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A303" s="3">
         <v>37130189</v>
       </c>
@@ -29285,7 +29297,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="304" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A304" s="3">
         <v>37130242</v>
       </c>
@@ -29373,7 +29385,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="305" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A305" s="3">
         <v>37130264</v>
       </c>
@@ -29467,7 +29479,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="306" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A306" s="3">
         <v>37130264</v>
       </c>
@@ -29561,7 +29573,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="307" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A307" s="3">
         <v>37130264</v>
       </c>
@@ -29655,7 +29667,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="308" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A308" s="3">
         <v>37130270</v>
       </c>
@@ -29738,7 +29750,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="309" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A309" s="3">
         <v>37130270</v>
       </c>
@@ -29821,7 +29833,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="310" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A310" s="3">
         <v>37130278</v>
       </c>
@@ -29910,7 +29922,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="311" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A311" s="3">
         <v>37130278</v>
       </c>
@@ -29995,7 +30007,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="312" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A312" s="3">
         <v>37130278</v>
       </c>
@@ -30083,7 +30095,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="313" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A313" s="3">
         <v>37130294</v>
       </c>
@@ -30207,7 +30219,7 @@
         <v>5274</v>
       </c>
     </row>
-    <row r="314" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A314" s="3">
         <v>37130294</v>
       </c>
@@ -30331,7 +30343,7 @@
         <v>5274</v>
       </c>
     </row>
-    <row r="315" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A315" s="3">
         <v>37130328</v>
       </c>
@@ -30450,7 +30462,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="316" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A316" s="3">
         <v>37130328</v>
       </c>
@@ -30569,7 +30581,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="317" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A317" s="3">
         <v>37130328</v>
       </c>
@@ -30687,7 +30699,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="318" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A318" s="3">
         <v>37130328</v>
       </c>
@@ -30805,7 +30817,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="319" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A319" s="3">
         <v>37130328</v>
       </c>
@@ -30923,7 +30935,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="320" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A320" s="3">
         <v>37130328</v>
       </c>
@@ -31041,7 +31053,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="321" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A321" s="3">
         <v>37130377</v>
       </c>
@@ -31166,7 +31178,7 @@
         <v>4664</v>
       </c>
     </row>
-    <row r="322" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A322" s="3">
         <v>37130382</v>
       </c>
@@ -31292,7 +31304,7 @@
         <v>5388</v>
       </c>
     </row>
-    <row r="323" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A323" s="3">
         <v>37130382</v>
       </c>
@@ -31418,7 +31430,7 @@
         <v>5388</v>
       </c>
     </row>
-    <row r="324" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A324" s="3">
         <v>37130382</v>
       </c>
@@ -31542,7 +31554,7 @@
         <v>5388</v>
       </c>
     </row>
-    <row r="325" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A325" s="3">
         <v>37130382</v>
       </c>
@@ -31666,7 +31678,7 @@
         <v>5388</v>
       </c>
     </row>
-    <row r="326" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A326" s="3">
         <v>37130382</v>
       </c>
@@ -31790,7 +31802,7 @@
         <v>5388</v>
       </c>
     </row>
-    <row r="327" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A327" s="3">
         <v>37130454</v>
       </c>
@@ -31912,7 +31924,7 @@
         <v>5200</v>
       </c>
     </row>
-    <row r="328" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A328" s="3">
         <v>37130454</v>
       </c>
@@ -32034,7 +32046,7 @@
         <v>5200</v>
       </c>
     </row>
-    <row r="329" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A329" s="3">
         <v>37130454</v>
       </c>
@@ -32155,7 +32167,7 @@
         <v>5200</v>
       </c>
     </row>
-    <row r="330" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A330" s="3">
         <v>37130485</v>
       </c>
@@ -32271,7 +32283,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="331" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A331" s="3">
         <v>37130485</v>
       </c>
@@ -32389,7 +32401,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="332" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A332" s="3">
         <v>37130485</v>
       </c>
@@ -32507,7 +32519,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="333" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A333" s="3">
         <v>37130485</v>
       </c>
@@ -32625,7 +32637,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="334" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A334" s="3">
         <v>37130485</v>
       </c>
@@ -32743,7 +32755,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="335" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A335" s="3">
         <v>37130485</v>
       </c>
@@ -32861,7 +32873,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="336" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A336" s="3">
         <v>37130501</v>
       </c>
@@ -32980,7 +32992,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="337" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A337" s="3">
         <v>37130501</v>
       </c>
@@ -33098,7 +33110,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="338" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A338" s="3">
         <v>37130504</v>
       </c>
@@ -33219,7 +33231,7 @@
         <v>5574</v>
       </c>
     </row>
-    <row r="339" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A339" s="3">
         <v>37130504</v>
       </c>
@@ -33340,7 +33352,7 @@
         <v>5574</v>
       </c>
     </row>
-    <row r="340" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A340" s="3">
         <v>37130524</v>
       </c>
@@ -33419,7 +33431,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="341" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A341" s="3">
         <v>37130567</v>
       </c>
@@ -33543,7 +33555,7 @@
         <v>5850</v>
       </c>
     </row>
-    <row r="342" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A342" s="3">
         <v>37130623</v>
       </c>
@@ -33661,7 +33673,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="343" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A343" s="3">
         <v>37130623</v>
       </c>
@@ -33779,7 +33791,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="344" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A344" s="3">
         <v>37130623</v>
       </c>
@@ -33897,7 +33909,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="345" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A345" s="3">
         <v>37130623</v>
       </c>
@@ -34015,7 +34027,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="346" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A346" s="3">
         <v>37130623</v>
       </c>
@@ -34133,7 +34145,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="347" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A347" s="3">
         <v>37130657</v>
       </c>
@@ -34208,7 +34220,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="348" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A348" s="3">
         <v>37130688</v>
       </c>
@@ -34330,7 +34342,7 @@
         <v>5391</v>
       </c>
     </row>
-    <row r="349" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A349" s="3">
         <v>37130688</v>
       </c>
@@ -34451,7 +34463,7 @@
         <v>5391</v>
       </c>
     </row>
-    <row r="350" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A350" s="3">
         <v>37130688</v>
       </c>
@@ -34572,7 +34584,7 @@
         <v>5391</v>
       </c>
     </row>
-    <row r="351" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A351" s="3">
         <v>37130775</v>
       </c>
@@ -34691,7 +34703,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="352" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A352" s="3">
         <v>37130775</v>
       </c>
@@ -34810,7 +34822,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="353" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A353" s="3">
         <v>37130775</v>
       </c>
@@ -34928,7 +34940,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="354" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A354" s="3">
         <v>37130778</v>
       </c>
@@ -34979,7 +34991,7 @@
         <v>37130778___1</v>
       </c>
     </row>
-    <row r="355" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A355" s="3">
         <v>37130807</v>
       </c>
@@ -35104,7 +35116,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="356" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A356" s="3">
         <v>37130807</v>
       </c>
@@ -35228,7 +35240,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="357" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A357" s="3">
         <v>37131375</v>
       </c>
@@ -35328,7 +35340,7 @@
         <v>4800</v>
       </c>
     </row>
-    <row r="358" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A358" s="3">
         <v>37133244</v>
       </c>
@@ -35449,7 +35461,7 @@
         <v>4750</v>
       </c>
     </row>
-    <row r="359" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A359" s="3">
         <v>37133745</v>
       </c>
@@ -35573,7 +35585,7 @@
         <v>5516</v>
       </c>
     </row>
-    <row r="360" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A360" s="3">
         <v>37133745</v>
       </c>
@@ -35697,7 +35709,7 @@
         <v>5516</v>
       </c>
     </row>
-    <row r="361" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A361" s="3">
         <v>37134233</v>
       </c>
@@ -35797,7 +35809,7 @@
         <v>4930</v>
       </c>
     </row>
-    <row r="362" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A362" s="3">
         <v>37134544</v>
       </c>
@@ -35897,7 +35909,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="363" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A363" s="3">
         <v>37134606</v>
       </c>
@@ -36015,7 +36027,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="364" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A364" s="3">
         <v>37136228</v>
       </c>
@@ -36133,7 +36145,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="365" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A365" s="3">
         <v>37136228</v>
       </c>
@@ -36251,7 +36263,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="366" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A366" s="3">
         <v>37136247</v>
       </c>
@@ -36372,7 +36384,7 @@
         <v>5172</v>
       </c>
     </row>
-    <row r="367" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A367" s="3">
         <v>37136248</v>
       </c>
@@ -36490,7 +36502,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="368" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A368" s="3">
         <v>37136248</v>
       </c>
@@ -36608,7 +36620,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="369" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A369" s="3">
         <v>37136248</v>
       </c>
@@ -36726,7 +36738,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="370" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A370" s="3">
         <v>37136277</v>
       </c>
@@ -36847,7 +36859,7 @@
         <v>5350</v>
       </c>
     </row>
-    <row r="371" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A371" s="3">
         <v>37136282</v>
       </c>
@@ -36931,7 +36943,7 @@
         <v>37136282___1</v>
       </c>
     </row>
-    <row r="372" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A372" s="3">
         <v>37136283</v>
       </c>
@@ -37052,7 +37064,7 @@
         <v>5258</v>
       </c>
     </row>
-    <row r="373" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A373" s="3">
         <v>37136283</v>
       </c>
@@ -37173,7 +37185,7 @@
         <v>5258</v>
       </c>
     </row>
-    <row r="374" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A374" s="3">
         <v>37136291</v>
       </c>
@@ -37291,7 +37303,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="375" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A375" s="3">
         <v>37136294</v>
       </c>
@@ -37414,7 +37426,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="376" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A376" s="3">
         <v>37136294</v>
       </c>
@@ -37537,7 +37549,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="377" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A377" s="3">
         <v>37136294</v>
       </c>
@@ -37660,7 +37672,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="378" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A378" s="3">
         <v>37136294</v>
       </c>
@@ -37784,7 +37796,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="379" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A379" s="3">
         <v>37136294</v>
       </c>
@@ -37908,7 +37920,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="380" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A380" s="3">
         <v>37136294</v>
       </c>
@@ -38032,7 +38044,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="381" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A381" s="3">
         <v>37136294</v>
       </c>
@@ -38156,7 +38168,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="382" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A382" s="3">
         <v>37136294</v>
       </c>
@@ -38280,7 +38292,7 @@
         <v>5439</v>
       </c>
     </row>
-    <row r="383" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A383" s="3">
         <v>37136299</v>
       </c>
@@ -38398,7 +38410,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="384" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="384" spans="1:39" x14ac:dyDescent="0.25">
       <c r="A384" s="3">
         <v>37136299</v>
       </c>
@@ -38516,7 +38528,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="385" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="385" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A385" s="3">
         <v>37136313</v>
       </c>
@@ -38640,7 +38652,7 @@
         <v>5293</v>
       </c>
     </row>
-    <row r="386" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="386" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A386" s="3">
         <v>37136313</v>
       </c>
@@ -38764,7 +38776,7 @@
         <v>5293</v>
       </c>
     </row>
-    <row r="387" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="387" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A387" s="3">
         <v>37136355</v>
       </c>
@@ -38882,13 +38894,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="388" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="388" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A388" s="3">
         <v>37136355</v>
       </c>
-      <c r="B388" s="3" t="str">
-        <f t="shared" si="50"/>
-        <v>08-   3W -3W</v>
+      <c r="B388" s="3" t="s">
+        <v>374</v>
       </c>
       <c r="C388" t="s">
         <v>352</v>
@@ -39000,7 +39011,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="389" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="389" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A389" s="4">
         <v>37136717</v>
       </c>
@@ -39117,7 +39128,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="390" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="390" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A390" s="3">
         <v>37136717</v>
       </c>
@@ -39234,7 +39245,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="391" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A391" s="3">
         <v>37137035</v>
       </c>
@@ -39352,7 +39363,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="392" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="392" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A392" s="3">
         <v>37137240</v>
       </c>
@@ -39451,7 +39462,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="393" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="393" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A393" s="3">
         <v>37138881</v>
       </c>
@@ -39569,7 +39580,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="394" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="394" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A394" s="4">
         <v>37140161</v>
       </c>
@@ -39580,7 +39591,7 @@
         <v>1</v>
       </c>
       <c r="D394" s="5" t="s">
-        <v>63</v>
+        <v>142</v>
       </c>
       <c r="E394" s="5">
         <v>11</v>
@@ -39679,14 +39690,14 @@
         <f t="shared" si="49"/>
         <v>37140161_08_1_1</v>
       </c>
-      <c r="AJ394" s="5" t="s">
-        <v>72</v>
+      <c r="AJ394" s="10" t="s">
+        <v>86</v>
       </c>
       <c r="AK394" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="395" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="395" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A395" s="3">
         <v>37140183</v>
       </c>
@@ -39773,7 +39784,7 @@
         <v>37140183___2</v>
       </c>
     </row>
-    <row r="396" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="396" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A396" s="4">
         <v>37140258</v>
       </c>
@@ -39890,7 +39901,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="397" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="397" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A397" s="3">
         <v>37140289</v>
       </c>
@@ -39977,7 +39988,7 @@
         <v>37140289___10</v>
       </c>
     </row>
-    <row r="398" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="398" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A398" s="3">
         <v>37140290</v>
       </c>
@@ -40064,7 +40075,7 @@
         <v>37140290___9</v>
       </c>
     </row>
-    <row r="399" spans="1:41" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:41" x14ac:dyDescent="0.25">
       <c r="A399" s="3">
         <v>37140291</v>
       </c>
@@ -40151,7 +40162,7 @@
         <v>37140291___5</v>
       </c>
     </row>
-    <row r="400" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="400" spans="1:41" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A400" s="4">
         <v>37140292</v>
       </c>
@@ -40268,7 +40279,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="401" spans="1:37" s="5" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="401" spans="1:37" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A401" s="4">
         <v>37140313</v>
       </c>
@@ -40395,7 +40406,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{406464DF-9C06-46D2-9215-AFFF9C8DD2FA}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>